<commit_message>
Complete P360 automation framework with API and export validation
</commit_message>
<xml_diff>
--- a/test-data/P360_TestCases.xlsx
+++ b/test-data/P360_TestCases.xlsx
@@ -486,7 +486,7 @@
         <v>PASS</v>
       </c>
     </row>
-    <row r="4" xml:space="preserve">
+    <row r="4">
       <c r="A4" t="str">
         <v>TC003</v>
       </c>
@@ -508,15 +508,11 @@
       <c r="G4" t="str">
         <v>Results should display</v>
       </c>
-      <c r="H4" t="str" xml:space="preserve">
-        <v xml:space="preserve">locator.waitFor: Timeout 90000ms exceeded.
-Call log:
-_x001b_[2m  - waiting for getByRole('main').locator('span.product-description').first() to be visible_x001b_[22m
-_x001b_[2m    179 × locator resolved to hidden &lt;span _ngcontent-ng-c804724162="" class="product-description ng-star-inserted"&gt;&lt;/span&gt;_x001b_[22m
-</v>
+      <c r="H4" t="str">
+        <v>Results displayed successfully for 4900005276</v>
       </c>
       <c r="I4" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance P360 automation with API logging, performance metrics, and Excel-driven catalog upload tests
</commit_message>
<xml_diff>
--- a/test-data/P360_TestCases.xlsx
+++ b/test-data/P360_TestCases.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:L4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -427,6 +427,15 @@
       <c r="I1" t="str">
         <v>Status</v>
       </c>
+      <c r="J1" t="str">
+        <v>GetProduct360SearchResults (ms)</v>
+      </c>
+      <c r="K1" t="str">
+        <v>LoadProduct360ViewV5 (ms)</v>
+      </c>
+      <c r="L1" t="str">
+        <v>ProductDetailPageLoad (ms)</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -456,6 +465,15 @@
       <c r="I2" t="str">
         <v>PASS</v>
       </c>
+      <c r="J2">
+        <v>3541</v>
+      </c>
+      <c r="K2">
+        <v>16675</v>
+      </c>
+      <c r="L2">
+        <v>61</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -485,6 +503,15 @@
       <c r="I3" t="str">
         <v>PASS</v>
       </c>
+      <c r="J3">
+        <v>1502</v>
+      </c>
+      <c r="K3">
+        <v>15644</v>
+      </c>
+      <c r="L3">
+        <v>50</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -514,10 +541,19 @@
       <c r="I4" t="str">
         <v>PASS</v>
       </c>
+      <c r="J4">
+        <v>1330</v>
+      </c>
+      <c r="K4">
+        <v>4391</v>
+      </c>
+      <c r="L4">
+        <v>37</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>